<commit_message>
feat: add Outlier Check sheet to Data Cleaning Log
</commit_message>
<xml_diff>
--- a/docs/Final Project/03_Data_Cleaning/Data_Cleaning_Log.xlsx
+++ b/docs/Final Project/03_Data_Cleaning/Data_Cleaning_Log.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaning Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outlier Check" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +45,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00366092"/>
+        <bgColor rgb="00366092"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -76,6 +83,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1129,4 +1140,220 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>IQR</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Upper Boundary</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Outliers Count</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Max Value</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Outlier %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Total Pembayaran</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>13675</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>42311.25</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>28636.25</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>85265.625</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>2073</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>3076000</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>10.99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>total_qty</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>2335</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>256</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>12.56%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Total Diskon</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>126</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>700000</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>0.67%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>total_weight_gr</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3550</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>2220</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>375000</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>11.77%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Perkiraan Ongkos Kirim</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>38000</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1669</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>624000</v>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>8.85%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>